<commit_message>
feat(gameconfig): update bgcoinweight values for game configuration
</commit_message>
<xml_diff>
--- a/assets/gamecfg002/bgcoinweight.xlsx
+++ b/assets/gamecfg002/bgcoinweight.xlsx
@@ -19,16 +19,16 @@
     <t>weight</t>
   </si>
   <si>
-    <t>1</t>
+    <t>10</t>
   </si>
   <si>
-    <t>2</t>
+    <t>20</t>
   </si>
   <si>
-    <t>5</t>
+    <t>50</t>
   </si>
   <si>
-    <t>10</t>
+    <t>100</t>
   </si>
 </sst>
 </file>
@@ -1427,7 +1427,7 @@
     </row>
     <row r="6" ht="15.35" customHeight="1">
       <c r="A6" s="7">
-        <v>25</v>
+        <v>250</v>
       </c>
       <c r="B6" s="8">
         <v>5</v>
@@ -1438,7 +1438,7 @@
     </row>
     <row r="7" ht="15.35" customHeight="1">
       <c r="A7" s="11">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="B7" s="12">
         <v>5</v>
@@ -1449,7 +1449,7 @@
     </row>
     <row r="8" ht="15.35" customHeight="1">
       <c r="A8" s="11">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="B8" s="12">
         <v>5</v>
@@ -1460,7 +1460,7 @@
     </row>
     <row r="9" ht="15.35" customHeight="1">
       <c r="A9" s="11">
-        <v>250</v>
+        <v>2500</v>
       </c>
       <c r="B9" s="12">
         <v>5</v>
@@ -1471,7 +1471,7 @@
     </row>
     <row r="10" ht="15.35" customHeight="1">
       <c r="A10" s="11">
-        <v>500</v>
+        <v>5000</v>
       </c>
       <c r="B10" s="12">
         <v>5</v>
@@ -1482,7 +1482,7 @@
     </row>
     <row r="11" ht="15.35" customHeight="1">
       <c r="A11" s="15">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="B11" s="16">
         <v>5</v>

</xml_diff>